<commit_message>
rate/hour now comes from wages sheet. And if employee is deleted from wages source data then it will be deleted from everthing but with a warning
</commit_message>
<xml_diff>
--- a/rick temp/project/Wages.xlsx
+++ b/rick temp/project/Wages.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmostert\Desktop\rick temp\project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADDDEF21-41CF-47A9-995E-0E897109A04A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A12E41E-78E0-46F6-82F1-21DF957A2F73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{51929737-26DB-4ED6-A5F0-52675FEF673F}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="232">
   <si>
     <t>CON009J</t>
   </si>
@@ -729,30 +729,6 @@
   </si>
   <si>
     <t>JobDescrip</t>
-  </si>
-  <si>
-    <t>OTHER001</t>
-  </si>
-  <si>
-    <t>Other</t>
-  </si>
-  <si>
-    <t>W0000064</t>
-  </si>
-  <si>
-    <t>C000158B</t>
-  </si>
-  <si>
-    <t>Mpendulo</t>
-  </si>
-  <si>
-    <t>OTHER002</t>
-  </si>
-  <si>
-    <t>Faizel Williams</t>
-  </si>
-  <si>
-    <t>Injection</t>
   </si>
 </sst>
 </file>
@@ -895,7 +871,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1073,12 +1049,6 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1242,9 +1212,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1600,7 +1569,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A71F74A-0F00-49D2-83C6-4054108D9CD0}">
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:E83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
@@ -3021,74 +2990,6 @@
         <v>72.849999999999994</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="B84" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="D84" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="E84" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A85" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="B85" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D85" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="E85" s="1">
-        <v>81.61</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A86" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="B86" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="C86" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D86" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="E86" s="1">
-        <v>66.930000000000007</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A87" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="B87" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="D87" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="E87" s="1">
-        <v>127.46</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>